<commit_message>
atualizacao dos dados do 2Q26 da GOOGL
</commit_message>
<xml_diff>
--- a/analise_eua/tecnologia/google/googl_indicators.xlsx
+++ b/analise_eua/tecnologia/google/googl_indicators.xlsx
@@ -592,10 +592,10 @@
         <v>2025</v>
       </c>
       <c r="B2" t="n">
-        <v>28.67</v>
+        <v>28.66</v>
       </c>
       <c r="C2" t="n">
-        <v>28.67</v>
+        <v>28.65</v>
       </c>
       <c r="D2" t="n">
         <v>3.49</v>
@@ -607,10 +607,10 @@
         <v>32.81</v>
       </c>
       <c r="G2" t="n">
-        <v>9.130000000000001</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="H2" t="n">
-        <v>3789642480</v>
+        <v>3787340440</v>
       </c>
       <c r="I2" t="n">
         <v>59291</v>
@@ -628,7 +628,7 @@
         <v>-0.16</v>
       </c>
       <c r="N2" t="n">
-        <v>25.68</v>
+        <v>25.67</v>
       </c>
       <c r="O2" t="n">
         <v>31.83</v>
@@ -687,13 +687,13 @@
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>23.19</v>
+        <v>23.17</v>
       </c>
       <c r="C3" t="n">
-        <v>23.18</v>
+        <v>23.16</v>
       </c>
       <c r="D3" t="n">
-        <v>4.31</v>
+        <v>4.32</v>
       </c>
       <c r="E3" t="n">
         <v>127701</v>
@@ -705,7 +705,7 @@
         <v>7.14</v>
       </c>
       <c r="H3" t="n">
-        <v>2321269170</v>
+        <v>2319914080</v>
       </c>
       <c r="I3" t="n">
         <v>25461</v>
@@ -723,7 +723,7 @@
         <v>-0.22</v>
       </c>
       <c r="N3" t="n">
-        <v>18.73</v>
+        <v>18.72</v>
       </c>
       <c r="O3" t="n">
         <v>30.8</v>
@@ -782,10 +782,10 @@
         <v>2023</v>
       </c>
       <c r="B4" t="n">
+        <v>23.7</v>
+      </c>
+      <c r="C4" t="n">
         <v>23.71</v>
-      </c>
-      <c r="C4" t="n">
-        <v>23.72</v>
       </c>
       <c r="D4" t="n">
         <v>4.22</v>
@@ -800,7 +800,7 @@
         <v>6.17</v>
       </c>
       <c r="H4" t="n">
-        <v>1749760200</v>
+        <v>1748749800</v>
       </c>
       <c r="I4" t="n">
         <v>28867</v>
@@ -818,7 +818,7 @@
         <v>-0.29</v>
       </c>
       <c r="N4" t="n">
-        <v>19.03</v>
+        <v>19.02</v>
       </c>
       <c r="O4" t="n">
         <v>26.04</v>
@@ -877,10 +877,10 @@
         <v>2022</v>
       </c>
       <c r="B5" t="n">
-        <v>19.06</v>
+        <v>19.05</v>
       </c>
       <c r="C5" t="n">
-        <v>19.07</v>
+        <v>19.05</v>
       </c>
       <c r="D5" t="n">
         <v>5.25</v>
@@ -895,7 +895,7 @@
         <v>4.46</v>
       </c>
       <c r="H5" t="n">
-        <v>1143143130</v>
+        <v>1142359350</v>
       </c>
       <c r="I5" t="n">
         <v>29977</v>
@@ -913,7 +913,7 @@
         <v>-0.33</v>
       </c>
       <c r="N5" t="n">
-        <v>13.61</v>
+        <v>13.6</v>
       </c>
       <c r="O5" t="n">
         <v>23.41</v>
@@ -972,13 +972,13 @@
         <v>2021</v>
       </c>
       <c r="B6" t="n">
-        <v>25.23</v>
+        <v>25.22</v>
       </c>
       <c r="C6" t="n">
-        <v>25.23</v>
+        <v>25.22</v>
       </c>
       <c r="D6" t="n">
-        <v>3.96</v>
+        <v>3.97</v>
       </c>
       <c r="E6" t="n">
         <v>90269</v>
@@ -990,7 +990,7 @@
         <v>7.62</v>
       </c>
       <c r="H6" t="n">
-        <v>1918291980</v>
+        <v>1917223740</v>
       </c>
       <c r="I6" t="n">
         <v>28508</v>
@@ -1008,7 +1008,7 @@
         <v>-0.44</v>
       </c>
       <c r="N6" t="n">
-        <v>22.48</v>
+        <v>22.47</v>
       </c>
       <c r="O6" t="n">
         <v>30.22</v>
@@ -1067,10 +1067,10 @@
         <v>2020</v>
       </c>
       <c r="B7" t="n">
-        <v>29.39</v>
+        <v>29.37</v>
       </c>
       <c r="C7" t="n">
-        <v>29.39</v>
+        <v>29.37</v>
       </c>
       <c r="D7" t="n">
         <v>3.4</v>
@@ -1082,10 +1082,10 @@
         <v>22.06</v>
       </c>
       <c r="G7" t="n">
-        <v>5.32</v>
+        <v>5.31</v>
       </c>
       <c r="H7" t="n">
-        <v>1183401324</v>
+        <v>1182720504</v>
       </c>
       <c r="I7" t="n">
         <v>26873</v>
@@ -1103,7 +1103,7 @@
         <v>-0.49</v>
       </c>
       <c r="N7" t="n">
-        <v>23.89</v>
+        <v>23.88</v>
       </c>
       <c r="O7" t="n">
         <v>18.09</v>
@@ -1162,13 +1162,13 @@
         <v>2019</v>
       </c>
       <c r="B8" t="n">
-        <v>26.79</v>
+        <v>26.77</v>
       </c>
       <c r="C8" t="n">
-        <v>26.79</v>
+        <v>26.77</v>
       </c>
       <c r="D8" t="n">
-        <v>3.73</v>
+        <v>3.74</v>
       </c>
       <c r="E8" t="n">
         <v>45087</v>
@@ -1177,10 +1177,10 @@
         <v>21.22</v>
       </c>
       <c r="G8" t="n">
-        <v>4.57</v>
+        <v>4.56</v>
       </c>
       <c r="H8" t="n">
-        <v>920049840.0000001</v>
+        <v>919495760</v>
       </c>
       <c r="I8" t="n">
         <v>16082</v>
@@ -1198,7 +1198,7 @@
         <v>-0.51</v>
       </c>
       <c r="N8" t="n">
-        <v>22.7</v>
+        <v>22.69</v>
       </c>
       <c r="O8" t="n">
         <v>17.05</v>
@@ -1257,10 +1257,10 @@
         <v>2018</v>
       </c>
       <c r="B9" t="n">
-        <v>23.44</v>
+        <v>23.43</v>
       </c>
       <c r="C9" t="n">
-        <v>23.44</v>
+        <v>23.42</v>
       </c>
       <c r="D9" t="n">
         <v>4.27</v>
@@ -1272,10 +1272,10 @@
         <v>22.46</v>
       </c>
       <c r="G9" t="n">
-        <v>4.06</v>
+        <v>4.05</v>
       </c>
       <c r="H9" t="n">
-        <v>720443096</v>
+        <v>720026012</v>
       </c>
       <c r="I9" t="n">
         <v>4012</v>
@@ -1293,7 +1293,7 @@
         <v>-0.59</v>
       </c>
       <c r="N9" t="n">
-        <v>23.94</v>
+        <v>23.93</v>
       </c>
       <c r="O9" t="n">
         <v>17.3</v>
@@ -1352,10 +1352,10 @@
         <v>2017</v>
       </c>
       <c r="B10" t="n">
-        <v>57.17</v>
+        <v>57.14</v>
       </c>
       <c r="C10" t="n">
-        <v>57.19</v>
+        <v>57.15</v>
       </c>
       <c r="D10" t="n">
         <v>1.75</v>
@@ -1367,10 +1367,10 @@
         <v>11.42</v>
       </c>
       <c r="G10" t="n">
-        <v>4.75</v>
+        <v>4.74</v>
       </c>
       <c r="H10" t="n">
-        <v>723941919.9999999</v>
+        <v>723526180</v>
       </c>
       <c r="I10" t="n">
         <v>3969</v>
@@ -1388,7 +1388,7 @@
         <v>-0.64</v>
       </c>
       <c r="N10" t="n">
-        <v>25.48</v>
+        <v>25.47</v>
       </c>
       <c r="O10" t="n">
         <v>8.300000000000001</v>
@@ -1453,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE17"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1610,94 +1610,94 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46112</v>
+        <v>46203</v>
       </c>
       <c r="B2" t="n">
-        <v>55.6</v>
+        <v>38.7</v>
       </c>
       <c r="C2" t="n">
-        <v>21.74</v>
+        <v>18.21</v>
       </c>
       <c r="D2" t="n">
-        <v>4.6</v>
+        <v>5.49</v>
       </c>
       <c r="E2" t="n">
-        <v>46178</v>
+        <v>47874</v>
       </c>
       <c r="F2" t="n">
-        <v>56.94</v>
+        <v>93.65000000000001</v>
       </c>
       <c r="G2" t="n">
-        <v>7.27</v>
+        <v>6.78</v>
       </c>
       <c r="H2" t="n">
-        <v>3479188440</v>
+        <v>4342402870</v>
       </c>
       <c r="I2" t="n">
-        <v>90484</v>
+        <v>112756</v>
       </c>
       <c r="J2" t="n">
-        <v>126840</v>
+        <v>242474</v>
       </c>
       <c r="K2" t="n">
-        <v>-36356</v>
+        <v>-129718</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.24</v>
+        <v>-0.78</v>
       </c>
       <c r="M2" t="n">
-        <v>-0.08</v>
+        <v>-0.2</v>
       </c>
       <c r="N2" t="n">
-        <v>22.77</v>
+        <v>26.75</v>
       </c>
       <c r="O2" t="n">
-        <v>33.48</v>
+        <v>37.15</v>
       </c>
       <c r="P2" t="n">
-        <v>16.86</v>
+        <v>11.53</v>
       </c>
       <c r="Q2" t="n">
-        <v>45790</v>
+        <v>39069</v>
       </c>
       <c r="R2" t="n">
-        <v>-63389</v>
+        <v>-82433</v>
       </c>
       <c r="S2" t="n">
-        <v>25077</v>
+        <v>61243</v>
       </c>
       <c r="T2" t="n">
-        <v>10116</v>
+        <v>-5855</v>
       </c>
       <c r="U2" t="n">
-        <v>35674</v>
+        <v>44924</v>
       </c>
       <c r="V2" t="n">
-        <v>77692</v>
+        <v>102802</v>
       </c>
       <c r="W2" t="n">
-        <v>17032</v>
+        <v>18219</v>
       </c>
       <c r="X2" t="n">
-        <v>137239</v>
+        <v>167012</v>
       </c>
       <c r="Y2" t="n">
-        <v>102565</v>
+        <v>217413</v>
       </c>
       <c r="Z2" t="n">
-        <v>137.25</v>
+        <v>173.17</v>
       </c>
       <c r="AA2" t="n">
-        <v>129929</v>
+        <v>214671</v>
       </c>
       <c r="AB2" t="n">
-        <v>35179</v>
+        <v>29454</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.21</v>
+        <v>0.22</v>
       </c>
       <c r="AD2" t="n">
-        <v>4.06</v>
+        <v>2.4</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
@@ -1705,658 +1705,658 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45930</v>
+        <v>46112</v>
       </c>
       <c r="B3" t="n">
-        <v>83.88</v>
+        <v>55.56</v>
       </c>
       <c r="C3" t="n">
-        <v>23.8</v>
+        <v>21.72</v>
       </c>
       <c r="D3" t="n">
-        <v>4.2</v>
+        <v>4.6</v>
       </c>
       <c r="E3" t="n">
-        <v>36839</v>
+        <v>46178</v>
       </c>
       <c r="F3" t="n">
-        <v>34.18</v>
+        <v>56.94</v>
       </c>
       <c r="G3" t="n">
-        <v>7.58</v>
+        <v>7.26</v>
       </c>
       <c r="H3" t="n">
-        <v>2934118220</v>
+        <v>3477131610</v>
       </c>
       <c r="I3" t="n">
-        <v>33713</v>
+        <v>90484</v>
       </c>
       <c r="J3" t="n">
-        <v>98496</v>
+        <v>126840</v>
       </c>
       <c r="K3" t="n">
-        <v>-64783</v>
+        <v>-36356</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.46</v>
+        <v>-0.24</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.17</v>
+        <v>-0.08</v>
       </c>
       <c r="N3" t="n">
-        <v>21.31</v>
+        <v>22.76</v>
       </c>
       <c r="O3" t="n">
-        <v>32.06</v>
+        <v>33.48</v>
       </c>
       <c r="P3" t="n">
-        <v>22.4</v>
+        <v>16.86</v>
       </c>
       <c r="Q3" t="n">
-        <v>48414</v>
+        <v>45790</v>
       </c>
       <c r="R3" t="n">
-        <v>-27777</v>
+        <v>-63389</v>
       </c>
       <c r="S3" t="n">
-        <v>-18383</v>
+        <v>25077</v>
       </c>
       <c r="T3" t="n">
-        <v>24461</v>
+        <v>10116</v>
       </c>
       <c r="U3" t="n">
-        <v>23953</v>
+        <v>35674</v>
       </c>
       <c r="V3" t="n">
-        <v>57576</v>
+        <v>77692</v>
       </c>
       <c r="W3" t="n">
-        <v>15151</v>
+        <v>17032</v>
       </c>
       <c r="X3" t="n">
-        <v>112538</v>
+        <v>137239</v>
       </c>
       <c r="Y3" t="n">
-        <v>74397</v>
+        <v>102565</v>
       </c>
       <c r="Z3" t="n">
-        <v>106.16</v>
+        <v>137.25</v>
       </c>
       <c r="AA3" t="n">
-        <v>91227</v>
+        <v>129929</v>
       </c>
       <c r="AB3" t="n">
-        <v>51651</v>
+        <v>35179</v>
       </c>
       <c r="AC3" t="n">
         <v>0.21</v>
       </c>
       <c r="AD3" t="n">
-        <v>7.25</v>
+        <v>4.06</v>
       </c>
       <c r="AE3" t="n">
-        <v>11504</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45838</v>
+        <v>45930</v>
       </c>
       <c r="B4" t="n">
-        <v>75.59</v>
+        <v>83.83</v>
       </c>
       <c r="C4" t="n">
-        <v>19.07</v>
+        <v>23.79</v>
       </c>
       <c r="D4" t="n">
-        <v>5.24</v>
+        <v>4.2</v>
       </c>
       <c r="E4" t="n">
-        <v>36269</v>
+        <v>36839</v>
       </c>
       <c r="F4" t="n">
-        <v>29.24</v>
+        <v>34.18</v>
       </c>
       <c r="G4" t="n">
-        <v>5.87</v>
+        <v>7.58</v>
       </c>
       <c r="H4" t="n">
-        <v>2131411260</v>
+        <v>2932426180</v>
       </c>
       <c r="I4" t="n">
-        <v>35559</v>
+        <v>33713</v>
       </c>
       <c r="J4" t="n">
-        <v>95148</v>
+        <v>98496</v>
       </c>
       <c r="K4" t="n">
-        <v>-59589</v>
+        <v>-64783</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.44</v>
+        <v>-0.46</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.16</v>
+        <v>-0.17</v>
       </c>
       <c r="N4" t="n">
-        <v>16.23</v>
+        <v>21.3</v>
       </c>
       <c r="O4" t="n">
-        <v>31.04</v>
+        <v>32.06</v>
       </c>
       <c r="P4" t="n">
-        <v>23.97</v>
+        <v>22.4</v>
       </c>
       <c r="Q4" t="n">
-        <v>27747</v>
+        <v>48414</v>
       </c>
       <c r="R4" t="n">
-        <v>-24544</v>
+        <v>-27777</v>
       </c>
       <c r="S4" t="n">
-        <v>-5832</v>
+        <v>-18383</v>
       </c>
       <c r="T4" t="n">
-        <v>5301</v>
+        <v>24461</v>
       </c>
       <c r="U4" t="n">
-        <v>22446</v>
+        <v>23953</v>
       </c>
       <c r="V4" t="n">
-        <v>48712</v>
+        <v>57576</v>
       </c>
       <c r="W4" t="n">
-        <v>13808</v>
+        <v>15151</v>
       </c>
       <c r="X4" t="n">
-        <v>100383</v>
+        <v>112538</v>
       </c>
       <c r="Y4" t="n">
-        <v>78906</v>
+        <v>74397</v>
       </c>
       <c r="Z4" t="n">
-        <v>116.16</v>
+        <v>106.16</v>
       </c>
       <c r="AA4" t="n">
-        <v>67211</v>
+        <v>91227</v>
       </c>
       <c r="AB4" t="n">
-        <v>38637</v>
+        <v>51651</v>
       </c>
       <c r="AC4" t="n">
         <v>0.21</v>
       </c>
       <c r="AD4" t="n">
-        <v>9.02</v>
+        <v>7.25</v>
       </c>
       <c r="AE4" t="n">
-        <v>13638</v>
+        <v>11504</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45747</v>
+        <v>45838</v>
       </c>
       <c r="B5" t="n">
-        <v>54.36</v>
+        <v>75.55</v>
       </c>
       <c r="C5" t="n">
-        <v>17.51</v>
+        <v>19.06</v>
       </c>
       <c r="D5" t="n">
-        <v>5.71</v>
+        <v>5.25</v>
       </c>
       <c r="E5" t="n">
-        <v>35093</v>
+        <v>36269</v>
       </c>
       <c r="F5" t="n">
-        <v>38.28</v>
+        <v>29.24</v>
       </c>
       <c r="G5" t="n">
-        <v>5.44</v>
+        <v>5.87</v>
       </c>
       <c r="H5" t="n">
-        <v>1877522130</v>
+        <v>2130199060</v>
       </c>
       <c r="I5" t="n">
-        <v>22564</v>
+        <v>35559</v>
       </c>
       <c r="J5" t="n">
-        <v>95328</v>
+        <v>95148</v>
       </c>
       <c r="K5" t="n">
-        <v>-72764</v>
+        <v>-59589</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.57</v>
+        <v>-0.44</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.21</v>
+        <v>-0.16</v>
       </c>
       <c r="N5" t="n">
-        <v>15.28</v>
+        <v>16.22</v>
       </c>
       <c r="O5" t="n">
-        <v>31.32</v>
+        <v>31.04</v>
       </c>
       <c r="P5" t="n">
-        <v>24.68</v>
+        <v>23.97</v>
       </c>
       <c r="Q5" t="n">
-        <v>36150</v>
+        <v>27747</v>
       </c>
       <c r="R5" t="n">
-        <v>-16194</v>
+        <v>-24544</v>
       </c>
       <c r="S5" t="n">
-        <v>-20201</v>
+        <v>-5832</v>
       </c>
       <c r="T5" t="n">
-        <v>18953</v>
+        <v>5301</v>
       </c>
       <c r="U5" t="n">
-        <v>17197</v>
+        <v>22446</v>
       </c>
       <c r="V5" t="n">
-        <v>39863</v>
+        <v>48712</v>
       </c>
       <c r="W5" t="n">
-        <v>13556</v>
+        <v>13808</v>
       </c>
       <c r="X5" t="n">
-        <v>89629</v>
+        <v>100383</v>
       </c>
       <c r="Y5" t="n">
-        <v>70398</v>
+        <v>78906</v>
       </c>
       <c r="Z5" t="n">
-        <v>97.53</v>
+        <v>116.16</v>
       </c>
       <c r="AA5" t="n">
-        <v>69099</v>
+        <v>67211</v>
       </c>
       <c r="AB5" t="n">
-        <v>53815</v>
+        <v>38637</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="AD5" t="n">
-        <v>7.05</v>
+        <v>9.02</v>
       </c>
       <c r="AE5" t="n">
-        <v>15068</v>
+        <v>13638</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45565</v>
+        <v>45747</v>
       </c>
       <c r="B6" t="n">
-        <v>77.05</v>
+        <v>54.32</v>
       </c>
       <c r="C6" t="n">
-        <v>21.93</v>
+        <v>17.5</v>
       </c>
       <c r="D6" t="n">
-        <v>4.56</v>
+        <v>5.71</v>
       </c>
       <c r="E6" t="n">
-        <v>32506</v>
+        <v>35093</v>
       </c>
       <c r="F6" t="n">
-        <v>29.8</v>
+        <v>38.28</v>
       </c>
       <c r="G6" t="n">
-        <v>6.45</v>
+        <v>5.43</v>
       </c>
       <c r="H6" t="n">
-        <v>2026621000</v>
+        <v>1876303830</v>
       </c>
       <c r="I6" t="n">
-        <v>23951</v>
+        <v>22564</v>
       </c>
       <c r="J6" t="n">
-        <v>93230</v>
+        <v>95328</v>
       </c>
       <c r="K6" t="n">
-        <v>-69279</v>
+        <v>-72764</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.59</v>
+        <v>-0.57</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.22</v>
+        <v>-0.21</v>
       </c>
       <c r="N6" t="n">
-        <v>17.83</v>
+        <v>15.27</v>
       </c>
       <c r="O6" t="n">
-        <v>29.69</v>
+        <v>31.32</v>
       </c>
       <c r="P6" t="n">
-        <v>25.81</v>
+        <v>24.68</v>
       </c>
       <c r="Q6" t="n">
-        <v>30698</v>
+        <v>36150</v>
       </c>
       <c r="R6" t="n">
-        <v>-18011</v>
+        <v>-16194</v>
       </c>
       <c r="S6" t="n">
-        <v>-20094</v>
+        <v>-20201</v>
       </c>
       <c r="T6" t="n">
-        <v>17637</v>
+        <v>18953</v>
       </c>
       <c r="U6" t="n">
-        <v>13061</v>
+        <v>17197</v>
       </c>
       <c r="V6" t="n">
-        <v>31537</v>
+        <v>39863</v>
       </c>
       <c r="W6" t="n">
-        <v>12447</v>
+        <v>13556</v>
       </c>
       <c r="X6" t="n">
-        <v>79005</v>
+        <v>89629</v>
       </c>
       <c r="Y6" t="n">
-        <v>76738</v>
+        <v>70398</v>
       </c>
       <c r="Z6" t="n">
-        <v>96.11</v>
+        <v>97.53</v>
       </c>
       <c r="AA6" t="n">
-        <v>56451</v>
+        <v>69099</v>
       </c>
       <c r="AB6" t="n">
-        <v>48846</v>
+        <v>53815</v>
       </c>
       <c r="AC6" t="n">
         <v>0.2</v>
       </c>
       <c r="AD6" t="n">
-        <v>9.33</v>
+        <v>7.05</v>
       </c>
       <c r="AE6" t="n">
-        <v>15291</v>
+        <v>15068</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45473</v>
+        <v>45565</v>
       </c>
       <c r="B7" t="n">
-        <v>94.52</v>
+        <v>77.01000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>26.48</v>
+        <v>21.91</v>
       </c>
       <c r="D7" t="n">
-        <v>3.78</v>
+        <v>4.56</v>
       </c>
       <c r="E7" t="n">
-        <v>31133</v>
+        <v>32506</v>
       </c>
       <c r="F7" t="n">
-        <v>27.87</v>
+        <v>29.8</v>
       </c>
       <c r="G7" t="n">
-        <v>7.42</v>
+        <v>6.45</v>
       </c>
       <c r="H7" t="n">
-        <v>2232354980</v>
+        <v>2025392000</v>
       </c>
       <c r="I7" t="n">
-        <v>24946</v>
+        <v>23951</v>
       </c>
       <c r="J7" t="n">
-        <v>100725</v>
+        <v>93230</v>
       </c>
       <c r="K7" t="n">
-        <v>-75779</v>
+        <v>-69279</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-0.59</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.25</v>
+        <v>-0.22</v>
       </c>
       <c r="N7" t="n">
-        <v>20.95</v>
+        <v>17.82</v>
       </c>
       <c r="O7" t="n">
-        <v>28.37</v>
+        <v>29.69</v>
       </c>
       <c r="P7" t="n">
-        <v>25.31</v>
+        <v>25.81</v>
       </c>
       <c r="Q7" t="n">
-        <v>26640</v>
+        <v>30698</v>
       </c>
       <c r="R7" t="n">
-        <v>-2781</v>
+        <v>-18011</v>
       </c>
       <c r="S7" t="n">
-        <v>-20889</v>
+        <v>-20094</v>
       </c>
       <c r="T7" t="n">
-        <v>13454</v>
+        <v>17637</v>
       </c>
       <c r="U7" t="n">
-        <v>13186</v>
+        <v>13061</v>
       </c>
       <c r="V7" t="n">
-        <v>26070</v>
+        <v>31537</v>
       </c>
       <c r="W7" t="n">
-        <v>11860</v>
+        <v>12447</v>
       </c>
       <c r="X7" t="n">
-        <v>71679</v>
+        <v>79005</v>
       </c>
       <c r="Y7" t="n">
-        <v>84082</v>
+        <v>76738</v>
       </c>
       <c r="Z7" t="n">
-        <v>97.16</v>
+        <v>96.11</v>
       </c>
       <c r="AA7" t="n">
-        <v>49916</v>
+        <v>56451</v>
       </c>
       <c r="AB7" t="n">
-        <v>47869</v>
+        <v>48846</v>
       </c>
       <c r="AC7" t="n">
         <v>0.2</v>
       </c>
       <c r="AD7" t="n">
-        <v>10.44</v>
+        <v>9.33</v>
       </c>
       <c r="AE7" t="n">
-        <v>15684</v>
+        <v>15291</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45382</v>
+        <v>45473</v>
       </c>
       <c r="B8" t="n">
-        <v>78.54000000000001</v>
+        <v>94.45999999999999</v>
       </c>
       <c r="C8" t="n">
-        <v>24.54</v>
+        <v>26.47</v>
       </c>
       <c r="D8" t="n">
-        <v>4.08</v>
+        <v>3.78</v>
       </c>
       <c r="E8" t="n">
-        <v>28885</v>
+        <v>31133</v>
       </c>
       <c r="F8" t="n">
-        <v>29.38</v>
+        <v>27.87</v>
       </c>
       <c r="G8" t="n">
-        <v>6.35</v>
+        <v>7.42</v>
       </c>
       <c r="H8" t="n">
-        <v>1858401350</v>
+        <v>2231120680</v>
       </c>
       <c r="I8" t="n">
-        <v>25185</v>
+        <v>24946</v>
       </c>
       <c r="J8" t="n">
-        <v>108090</v>
+        <v>100725</v>
       </c>
       <c r="K8" t="n">
-        <v>-82905</v>
+        <v>-75779</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.83</v>
+        <v>-0.6899999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>-0.28</v>
+        <v>-0.25</v>
       </c>
       <c r="N8" t="n">
-        <v>19.51</v>
+        <v>20.94</v>
       </c>
       <c r="O8" t="n">
-        <v>26.22</v>
+        <v>28.37</v>
       </c>
       <c r="P8" t="n">
-        <v>23.02</v>
+        <v>25.31</v>
       </c>
       <c r="Q8" t="n">
-        <v>28848</v>
+        <v>26640</v>
       </c>
       <c r="R8" t="n">
-        <v>-8564</v>
+        <v>-2781</v>
       </c>
       <c r="S8" t="n">
-        <v>-19714</v>
+        <v>-20889</v>
       </c>
       <c r="T8" t="n">
-        <v>16836</v>
+        <v>13454</v>
       </c>
       <c r="U8" t="n">
-        <v>12012</v>
+        <v>13186</v>
       </c>
       <c r="V8" t="n">
-        <v>19821</v>
+        <v>26070</v>
       </c>
       <c r="W8" t="n">
-        <v>11903</v>
+        <v>11860</v>
       </c>
       <c r="X8" t="n">
-        <v>65038</v>
+        <v>71679</v>
       </c>
       <c r="Y8" t="n">
-        <v>88474</v>
+        <v>84082</v>
       </c>
       <c r="Z8" t="n">
-        <v>91.62</v>
+        <v>97.16</v>
       </c>
       <c r="AA8" t="n">
-        <v>53485</v>
+        <v>49916</v>
       </c>
       <c r="AB8" t="n">
-        <v>50059</v>
+        <v>47869</v>
       </c>
       <c r="AC8" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="AD8" t="n">
-        <v>0</v>
+        <v>10.44</v>
       </c>
       <c r="AE8" t="n">
-        <v>15696</v>
+        <v>15684</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45199</v>
+        <v>45382</v>
       </c>
       <c r="B9" t="n">
-        <v>82.93000000000001</v>
+        <v>78.48999999999999</v>
       </c>
       <c r="C9" t="n">
-        <v>24.67</v>
+        <v>24.52</v>
       </c>
       <c r="D9" t="n">
-        <v>4.05</v>
+        <v>4.08</v>
       </c>
       <c r="E9" t="n">
-        <v>25014</v>
+        <v>28885</v>
       </c>
       <c r="F9" t="n">
-        <v>25.67</v>
+        <v>29.38</v>
       </c>
       <c r="G9" t="n">
-        <v>5.98</v>
+        <v>6.34</v>
       </c>
       <c r="H9" t="n">
-        <v>1632887990</v>
+        <v>1857284000</v>
       </c>
       <c r="I9" t="n">
-        <v>26331</v>
+        <v>25185</v>
       </c>
       <c r="J9" t="n">
-        <v>119935</v>
+        <v>108090</v>
       </c>
       <c r="K9" t="n">
-        <v>-93604</v>
+        <v>-82905</v>
       </c>
       <c r="L9" t="n">
-        <v>-1.02</v>
+        <v>-0.83</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.34</v>
+        <v>-0.28</v>
       </c>
       <c r="N9" t="n">
-        <v>18.83</v>
+        <v>19.5</v>
       </c>
       <c r="O9" t="n">
-        <v>24.53</v>
+        <v>26.22</v>
       </c>
       <c r="P9" t="n">
-        <v>22.44</v>
+        <v>23.02</v>
       </c>
       <c r="Q9" t="n">
-        <v>30656</v>
+        <v>28848</v>
       </c>
       <c r="R9" t="n">
-        <v>-7150</v>
+        <v>-8564</v>
       </c>
       <c r="S9" t="n">
-        <v>-18382</v>
+        <v>-19714</v>
       </c>
       <c r="T9" t="n">
-        <v>22601</v>
+        <v>16836</v>
       </c>
       <c r="U9" t="n">
-        <v>8055</v>
+        <v>12012</v>
       </c>
       <c r="V9" t="n">
-        <v>14565</v>
+        <v>19821</v>
       </c>
       <c r="W9" t="n">
-        <v>11258</v>
+        <v>11903</v>
       </c>
       <c r="X9" t="n">
-        <v>58152</v>
+        <v>65038</v>
       </c>
       <c r="Y9" t="n">
-        <v>90015</v>
+        <v>88474</v>
       </c>
       <c r="Z9" t="n">
-        <v>86.09</v>
+        <v>91.62</v>
       </c>
       <c r="AA9" t="n">
-        <v>51749</v>
+        <v>53485</v>
       </c>
       <c r="AB9" t="n">
-        <v>57929</v>
+        <v>50059</v>
       </c>
       <c r="AC9" t="n">
         <v>0</v>
@@ -2365,42 +2365,42 @@
         <v>0</v>
       </c>
       <c r="AE9" t="n">
-        <v>15787</v>
+        <v>15696</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45107</v>
+        <v>45199</v>
       </c>
       <c r="B10" t="n">
-        <v>81.88</v>
+        <v>82.88</v>
       </c>
       <c r="C10" t="n">
-        <v>7.48</v>
+        <v>24.66</v>
       </c>
       <c r="D10" t="n">
-        <v>13.38</v>
+        <v>4.06</v>
       </c>
       <c r="E10" t="n">
-        <v>25117</v>
+        <v>25014</v>
       </c>
       <c r="F10" t="n">
-        <v>24.62</v>
+        <v>25.67</v>
       </c>
       <c r="G10" t="n">
-        <v>5.63</v>
+        <v>5.97</v>
       </c>
       <c r="H10" t="n">
-        <v>1503944960</v>
+        <v>1631881510</v>
       </c>
       <c r="I10" t="n">
-        <v>26451</v>
+        <v>26331</v>
       </c>
       <c r="J10" t="n">
-        <v>118332</v>
+        <v>119935</v>
       </c>
       <c r="K10" t="n">
-        <v>-91881</v>
+        <v>-93604</v>
       </c>
       <c r="L10" t="n">
         <v>-1.02</v>
@@ -2409,49 +2409,49 @@
         <v>-0.34</v>
       </c>
       <c r="N10" t="n">
-        <v>17.77</v>
+        <v>18.82</v>
       </c>
       <c r="O10" t="n">
-        <v>23.71</v>
+        <v>24.53</v>
       </c>
       <c r="P10" t="n">
-        <v>21.74</v>
+        <v>22.44</v>
       </c>
       <c r="Q10" t="n">
-        <v>28666</v>
+        <v>30656</v>
       </c>
       <c r="R10" t="n">
-        <v>-10800</v>
+        <v>-7150</v>
       </c>
       <c r="S10" t="n">
-        <v>-17835</v>
+        <v>-18382</v>
       </c>
       <c r="T10" t="n">
-        <v>21778</v>
+        <v>22601</v>
       </c>
       <c r="U10" t="n">
-        <v>6888</v>
+        <v>8055</v>
       </c>
       <c r="V10" t="n">
-        <v>13311</v>
+        <v>14565</v>
       </c>
       <c r="W10" t="n">
-        <v>10588</v>
+        <v>11258</v>
       </c>
       <c r="X10" t="n">
-        <v>55481</v>
+        <v>58152</v>
       </c>
       <c r="Y10" t="n">
-        <v>91079</v>
+        <v>90015</v>
       </c>
       <c r="Z10" t="n">
-        <v>86.11999999999999</v>
+        <v>86.09</v>
       </c>
       <c r="AA10" t="n">
-        <v>49354</v>
+        <v>51749</v>
       </c>
       <c r="AB10" t="n">
-        <v>50811</v>
+        <v>57929</v>
       </c>
       <c r="AC10" t="n">
         <v>0</v>
@@ -2460,93 +2460,93 @@
         <v>0</v>
       </c>
       <c r="AE10" t="n">
-        <v>14969</v>
+        <v>15787</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45016</v>
+        <v>45107</v>
       </c>
       <c r="B11" t="n">
-        <v>87.36</v>
+        <v>81.83</v>
       </c>
       <c r="C11" t="n">
-        <v>2.62</v>
+        <v>7.47</v>
       </c>
       <c r="D11" t="n">
-        <v>38.23</v>
+        <v>13.38</v>
       </c>
       <c r="E11" t="n">
-        <v>20475</v>
+        <v>25117</v>
       </c>
       <c r="F11" t="n">
-        <v>21.57</v>
+        <v>24.62</v>
       </c>
       <c r="G11" t="n">
-        <v>5.04</v>
+        <v>5.63</v>
       </c>
       <c r="H11" t="n">
-        <v>1314909280</v>
+        <v>1503058200</v>
       </c>
       <c r="I11" t="n">
-        <v>26496</v>
+        <v>26451</v>
       </c>
       <c r="J11" t="n">
-        <v>115102</v>
+        <v>118332</v>
       </c>
       <c r="K11" t="n">
-        <v>-88606</v>
+        <v>-91881</v>
       </c>
       <c r="L11" t="n">
-        <v>-1</v>
+        <v>-1.02</v>
       </c>
       <c r="M11" t="n">
         <v>-0.34</v>
       </c>
       <c r="N11" t="n">
-        <v>15.88</v>
+        <v>17.76</v>
       </c>
       <c r="O11" t="n">
-        <v>23.53</v>
+        <v>23.71</v>
       </c>
       <c r="P11" t="n">
-        <v>21.96</v>
+        <v>21.74</v>
       </c>
       <c r="Q11" t="n">
-        <v>23509</v>
+        <v>28666</v>
       </c>
       <c r="R11" t="n">
-        <v>-2946</v>
+        <v>-10800</v>
       </c>
       <c r="S11" t="n">
-        <v>-16568</v>
+        <v>-17835</v>
       </c>
       <c r="T11" t="n">
-        <v>17220</v>
+        <v>21778</v>
       </c>
       <c r="U11" t="n">
-        <v>6289</v>
+        <v>6888</v>
       </c>
       <c r="V11" t="n">
-        <v>15897</v>
+        <v>13311</v>
       </c>
       <c r="W11" t="n">
-        <v>11468</v>
+        <v>10588</v>
       </c>
       <c r="X11" t="n">
-        <v>56598</v>
+        <v>55481</v>
       </c>
       <c r="Y11" t="n">
-        <v>93131</v>
+        <v>91079</v>
       </c>
       <c r="Z11" t="n">
-        <v>90.44</v>
+        <v>86.11999999999999</v>
       </c>
       <c r="AA11" t="n">
-        <v>43968</v>
+        <v>49354</v>
       </c>
       <c r="AB11" t="n">
-        <v>44882</v>
+        <v>50811</v>
       </c>
       <c r="AC11" t="n">
         <v>0</v>
@@ -2555,93 +2555,93 @@
         <v>0</v>
       </c>
       <c r="AE11" t="n">
-        <v>14557</v>
+        <v>14969</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>44834</v>
+        <v>45016</v>
       </c>
       <c r="B12" t="n">
-        <v>88.79000000000001</v>
+        <v>87.31</v>
       </c>
       <c r="C12" t="n">
-        <v>1.42</v>
+        <v>2.61</v>
       </c>
       <c r="D12" t="n">
-        <v>70.19</v>
+        <v>38.25</v>
       </c>
       <c r="E12" t="n">
-        <v>21068</v>
+        <v>20475</v>
       </c>
       <c r="F12" t="n">
-        <v>20.13</v>
+        <v>21.57</v>
       </c>
       <c r="G12" t="n">
-        <v>4.87</v>
+        <v>5.04</v>
       </c>
       <c r="H12" t="n">
-        <v>1235017660</v>
+        <v>1314142420</v>
       </c>
       <c r="I12" t="n">
-        <v>26637</v>
+        <v>26496</v>
       </c>
       <c r="J12" t="n">
-        <v>116259</v>
+        <v>115102</v>
       </c>
       <c r="K12" t="n">
-        <v>-89622</v>
+        <v>-88606</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.97</v>
+        <v>-1</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.35</v>
+        <v>-0.34</v>
       </c>
       <c r="N12" t="n">
-        <v>14.4</v>
+        <v>15.87</v>
       </c>
       <c r="O12" t="n">
-        <v>25.74</v>
+        <v>23.53</v>
       </c>
       <c r="P12" t="n">
-        <v>23.46</v>
+        <v>21.96</v>
       </c>
       <c r="Q12" t="n">
-        <v>23353</v>
+        <v>23509</v>
       </c>
       <c r="R12" t="n">
-        <v>-833</v>
+        <v>-2946</v>
       </c>
       <c r="S12" t="n">
-        <v>-18097</v>
+        <v>-16568</v>
       </c>
       <c r="T12" t="n">
-        <v>16077</v>
+        <v>17220</v>
       </c>
       <c r="U12" t="n">
-        <v>7276</v>
+        <v>6289</v>
       </c>
       <c r="V12" t="n">
-        <v>16402</v>
+        <v>15897</v>
       </c>
       <c r="W12" t="n">
-        <v>10273</v>
+        <v>11468</v>
       </c>
       <c r="X12" t="n">
-        <v>53329</v>
+        <v>56598</v>
       </c>
       <c r="Y12" t="n">
-        <v>100130</v>
+        <v>93131</v>
       </c>
       <c r="Z12" t="n">
-        <v>82.82000000000001</v>
+        <v>90.44</v>
       </c>
       <c r="AA12" t="n">
-        <v>46688</v>
+        <v>43968</v>
       </c>
       <c r="AB12" t="n">
-        <v>49066</v>
+        <v>44882</v>
       </c>
       <c r="AC12" t="n">
         <v>0</v>
@@ -2650,93 +2650,93 @@
         <v>0</v>
       </c>
       <c r="AE12" t="n">
-        <v>15392</v>
+        <v>14557</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>44742</v>
+        <v>44834</v>
       </c>
       <c r="B13" t="n">
-        <v>177.39</v>
+        <v>88.73</v>
       </c>
       <c r="C13" t="n">
-        <v>23.19</v>
+        <v>1.42</v>
       </c>
       <c r="D13" t="n">
-        <v>4.31</v>
+        <v>70.23999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>23151</v>
+        <v>21068</v>
       </c>
       <c r="F13" t="n">
-        <v>22.96</v>
+        <v>20.13</v>
       </c>
       <c r="G13" t="n">
-        <v>11.11</v>
+        <v>4.87</v>
       </c>
       <c r="H13" t="n">
-        <v>2838566620</v>
+        <v>1234236580</v>
       </c>
       <c r="I13" t="n">
-        <v>26431</v>
+        <v>26637</v>
       </c>
       <c r="J13" t="n">
-        <v>124997</v>
+        <v>116259</v>
       </c>
       <c r="K13" t="n">
-        <v>-98566</v>
+        <v>-89622</v>
       </c>
       <c r="L13" t="n">
-        <v>-1.06</v>
+        <v>-0.97</v>
       </c>
       <c r="M13" t="n">
-        <v>-0.39</v>
+        <v>-0.35</v>
       </c>
       <c r="N13" t="n">
-        <v>31.57</v>
+        <v>14.39</v>
       </c>
       <c r="O13" t="n">
-        <v>27.37</v>
+        <v>25.74</v>
       </c>
       <c r="P13" t="n">
-        <v>23.72</v>
+        <v>23.46</v>
       </c>
       <c r="Q13" t="n">
-        <v>19422</v>
+        <v>23353</v>
       </c>
       <c r="R13" t="n">
-        <v>-4187</v>
+        <v>-833</v>
       </c>
       <c r="S13" t="n">
-        <v>-17817</v>
+        <v>-18097</v>
       </c>
       <c r="T13" t="n">
-        <v>12594</v>
+        <v>16077</v>
       </c>
       <c r="U13" t="n">
-        <v>6828</v>
+        <v>7276</v>
       </c>
       <c r="V13" t="n">
-        <v>15825</v>
+        <v>16402</v>
       </c>
       <c r="W13" t="n">
-        <v>9841</v>
+        <v>10273</v>
       </c>
       <c r="X13" t="n">
-        <v>50154</v>
+        <v>53329</v>
       </c>
       <c r="Y13" t="n">
-        <v>111017</v>
+        <v>100130</v>
       </c>
       <c r="Z13" t="n">
-        <v>84.56</v>
+        <v>82.82000000000001</v>
       </c>
       <c r="AA13" t="n">
-        <v>46272</v>
+        <v>46688</v>
       </c>
       <c r="AB13" t="n">
-        <v>45087</v>
+        <v>49066</v>
       </c>
       <c r="AC13" t="n">
         <v>0</v>
@@ -2745,93 +2745,93 @@
         <v>0</v>
       </c>
       <c r="AE13" t="n">
-        <v>15197</v>
+        <v>15392</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>44651</v>
+        <v>44742</v>
       </c>
       <c r="B14" t="n">
-        <v>110.8</v>
+        <v>177.29</v>
       </c>
       <c r="C14" t="n">
-        <v>25.62</v>
+        <v>23.18</v>
       </c>
       <c r="D14" t="n">
-        <v>3.9</v>
+        <v>4.31</v>
       </c>
       <c r="E14" t="n">
-        <v>23685</v>
+        <v>23151</v>
       </c>
       <c r="F14" t="n">
-        <v>24.17</v>
+        <v>22.96</v>
       </c>
       <c r="G14" t="n">
-        <v>7.17</v>
+        <v>11.11</v>
       </c>
       <c r="H14" t="n">
-        <v>1821144962</v>
+        <v>2836990660</v>
       </c>
       <c r="I14" t="n">
-        <v>26154</v>
+        <v>26431</v>
       </c>
       <c r="J14" t="n">
-        <v>133970</v>
+        <v>124997</v>
       </c>
       <c r="K14" t="n">
-        <v>-107816</v>
+        <v>-98566</v>
       </c>
       <c r="L14" t="n">
-        <v>-1.21</v>
+        <v>-1.06</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.42</v>
+        <v>-0.39</v>
       </c>
       <c r="N14" t="n">
-        <v>21.71</v>
+        <v>31.55</v>
       </c>
       <c r="O14" t="n">
-        <v>28.28</v>
+        <v>27.37</v>
       </c>
       <c r="P14" t="n">
-        <v>22.66</v>
+        <v>23.72</v>
       </c>
       <c r="Q14" t="n">
-        <v>25106</v>
+        <v>19422</v>
       </c>
       <c r="R14" t="n">
-        <v>-9051</v>
+        <v>-4187</v>
       </c>
       <c r="S14" t="n">
-        <v>-16214</v>
+        <v>-17817</v>
       </c>
       <c r="T14" t="n">
-        <v>15320</v>
+        <v>12594</v>
       </c>
       <c r="U14" t="n">
-        <v>9786</v>
+        <v>6828</v>
       </c>
       <c r="V14" t="n">
-        <v>16112</v>
+        <v>15825</v>
       </c>
       <c r="W14" t="n">
-        <v>9119</v>
+        <v>9841</v>
       </c>
       <c r="X14" t="n">
-        <v>48085</v>
+        <v>50154</v>
       </c>
       <c r="Y14" t="n">
-        <v>115905</v>
+        <v>111017</v>
       </c>
       <c r="Z14" t="n">
-        <v>77.62</v>
+        <v>84.56</v>
       </c>
       <c r="AA14" t="n">
-        <v>53403</v>
+        <v>46272</v>
       </c>
       <c r="AB14" t="n">
-        <v>49469</v>
+        <v>45087</v>
       </c>
       <c r="AC14" t="n">
         <v>0</v>
@@ -2840,93 +2840,93 @@
         <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>13300</v>
+        <v>15197</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>44469</v>
+        <v>44651</v>
       </c>
       <c r="B15" t="n">
-        <v>93.23</v>
+        <v>110.74</v>
       </c>
       <c r="C15" t="n">
-        <v>26.7</v>
+        <v>25.61</v>
       </c>
       <c r="D15" t="n">
-        <v>3.75</v>
+        <v>3.9</v>
       </c>
       <c r="E15" t="n">
-        <v>24116</v>
+        <v>23685</v>
       </c>
       <c r="F15" t="n">
-        <v>29.08</v>
+        <v>24.17</v>
       </c>
       <c r="G15" t="n">
-        <v>7.22</v>
+        <v>7.17</v>
       </c>
       <c r="H15" t="n">
-        <v>1765329216</v>
+        <v>1820088690</v>
       </c>
       <c r="I15" t="n">
-        <v>25759</v>
+        <v>26154</v>
       </c>
       <c r="J15" t="n">
-        <v>142003</v>
+        <v>133970</v>
       </c>
       <c r="K15" t="n">
-        <v>-116244</v>
+        <v>-107816</v>
       </c>
       <c r="L15" t="n">
-        <v>-1.46</v>
+        <v>-1.21</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.48</v>
+        <v>-0.42</v>
       </c>
       <c r="N15" t="n">
-        <v>23.62</v>
+        <v>21.7</v>
       </c>
       <c r="O15" t="n">
-        <v>27.25</v>
+        <v>28.28</v>
       </c>
       <c r="P15" t="n">
-        <v>20.34</v>
+        <v>22.66</v>
       </c>
       <c r="Q15" t="n">
-        <v>25539</v>
+        <v>25106</v>
       </c>
       <c r="R15" t="n">
-        <v>-10050</v>
+        <v>-9051</v>
       </c>
       <c r="S15" t="n">
-        <v>-15254</v>
+        <v>-16214</v>
       </c>
       <c r="T15" t="n">
-        <v>18720</v>
+        <v>15320</v>
       </c>
       <c r="U15" t="n">
-        <v>6819</v>
+        <v>9786</v>
       </c>
       <c r="V15" t="n">
-        <v>12034</v>
+        <v>16112</v>
       </c>
       <c r="W15" t="n">
-        <v>7694</v>
+        <v>9119</v>
       </c>
       <c r="X15" t="n">
-        <v>41744</v>
+        <v>48085</v>
       </c>
       <c r="Y15" t="n">
-        <v>122328</v>
+        <v>115905</v>
       </c>
       <c r="Z15" t="n">
-        <v>73.15000000000001</v>
+        <v>77.62</v>
       </c>
       <c r="AA15" t="n">
-        <v>64804</v>
+        <v>53403</v>
       </c>
       <c r="AB15" t="n">
-        <v>45349</v>
+        <v>49469</v>
       </c>
       <c r="AC15" t="n">
         <v>0</v>
@@ -2935,93 +2935,93 @@
         <v>0</v>
       </c>
       <c r="AE15" t="n">
-        <v>12610</v>
+        <v>13300</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>44377</v>
+        <v>44469</v>
       </c>
       <c r="B16" t="n">
-        <v>87.45</v>
+        <v>93.17</v>
       </c>
       <c r="C16" t="n">
-        <v>29.87</v>
+        <v>26.68</v>
       </c>
       <c r="D16" t="n">
-        <v>3.35</v>
+        <v>3.75</v>
       </c>
       <c r="E16" t="n">
-        <v>22091</v>
+        <v>24116</v>
       </c>
       <c r="F16" t="n">
-        <v>29.94</v>
+        <v>29.08</v>
       </c>
       <c r="G16" t="n">
-        <v>6.82</v>
+        <v>7.21</v>
       </c>
       <c r="H16" t="n">
-        <v>1620087328</v>
+        <v>1764264000</v>
       </c>
       <c r="I16" t="n">
-        <v>25947</v>
+        <v>25759</v>
       </c>
       <c r="J16" t="n">
-        <v>135863</v>
+        <v>142003</v>
       </c>
       <c r="K16" t="n">
-        <v>-109916</v>
+        <v>-116244</v>
       </c>
       <c r="L16" t="n">
-        <v>-1.69</v>
+        <v>-1.46</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.46</v>
+        <v>-0.48</v>
       </c>
       <c r="N16" t="n">
-        <v>26.57</v>
+        <v>23.6</v>
       </c>
       <c r="O16" t="n">
-        <v>23.01</v>
+        <v>27.25</v>
       </c>
       <c r="P16" t="n">
-        <v>16.38</v>
+        <v>20.34</v>
       </c>
       <c r="Q16" t="n">
-        <v>21890</v>
+        <v>25539</v>
       </c>
       <c r="R16" t="n">
-        <v>-9074</v>
+        <v>-10050</v>
       </c>
       <c r="S16" t="n">
-        <v>-15991</v>
+        <v>-15254</v>
       </c>
       <c r="T16" t="n">
-        <v>16394</v>
+        <v>18720</v>
       </c>
       <c r="U16" t="n">
-        <v>5496</v>
+        <v>6819</v>
       </c>
       <c r="V16" t="n">
-        <v>10513</v>
+        <v>12034</v>
       </c>
       <c r="W16" t="n">
-        <v>7675</v>
+        <v>7694</v>
       </c>
       <c r="X16" t="n">
-        <v>39404</v>
+        <v>41744</v>
       </c>
       <c r="Y16" t="n">
-        <v>119956</v>
+        <v>122328</v>
       </c>
       <c r="Z16" t="n">
-        <v>92.45999999999999</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="AA16" t="n">
-        <v>52344</v>
+        <v>64804</v>
       </c>
       <c r="AB16" t="n">
-        <v>33986</v>
+        <v>45349</v>
       </c>
       <c r="AC16" t="n">
         <v>0</v>
@@ -3030,101 +3030,196 @@
         <v>0</v>
       </c>
       <c r="AE16" t="n">
-        <v>12796</v>
+        <v>12610</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
+        <v>44377</v>
+      </c>
+      <c r="B17" t="n">
+        <v>87.40000000000001</v>
+      </c>
+      <c r="C17" t="n">
+        <v>29.85</v>
+      </c>
+      <c r="D17" t="n">
+        <v>3.35</v>
+      </c>
+      <c r="E17" t="n">
+        <v>22091</v>
+      </c>
+      <c r="F17" t="n">
+        <v>29.94</v>
+      </c>
+      <c r="G17" t="n">
+        <v>6.82</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1619150784</v>
+      </c>
+      <c r="I17" t="n">
+        <v>25947</v>
+      </c>
+      <c r="J17" t="n">
+        <v>135863</v>
+      </c>
+      <c r="K17" t="n">
+        <v>-109916</v>
+      </c>
+      <c r="L17" t="n">
+        <v>-1.69</v>
+      </c>
+      <c r="M17" t="n">
+        <v>-0.46</v>
+      </c>
+      <c r="N17" t="n">
+        <v>26.55</v>
+      </c>
+      <c r="O17" t="n">
+        <v>23.01</v>
+      </c>
+      <c r="P17" t="n">
+        <v>16.38</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>21890</v>
+      </c>
+      <c r="R17" t="n">
+        <v>-9074</v>
+      </c>
+      <c r="S17" t="n">
+        <v>-15991</v>
+      </c>
+      <c r="T17" t="n">
+        <v>16394</v>
+      </c>
+      <c r="U17" t="n">
+        <v>5496</v>
+      </c>
+      <c r="V17" t="n">
+        <v>10513</v>
+      </c>
+      <c r="W17" t="n">
+        <v>7675</v>
+      </c>
+      <c r="X17" t="n">
+        <v>39404</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>119956</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>92.45999999999999</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>52344</v>
+      </c>
+      <c r="AB17" t="n">
+        <v>33986</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE17" t="n">
+        <v>12796</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>44286</v>
       </c>
-      <c r="B17" t="n">
-        <v>76.81</v>
-      </c>
-      <c r="C17" t="n">
-        <v>32.29</v>
-      </c>
-      <c r="D17" t="n">
+      <c r="B18" t="n">
+        <v>76.76000000000001</v>
+      </c>
+      <c r="C18" t="n">
+        <v>32.27</v>
+      </c>
+      <c r="D18" t="n">
         <v>3.1</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E18" t="n">
         <v>18962</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F18" t="n">
         <v>32.41</v>
       </c>
-      <c r="G17" t="n">
-        <v>5.99</v>
-      </c>
-      <c r="H17" t="n">
-        <v>1377138832</v>
-      </c>
-      <c r="I17" t="n">
+      <c r="G18" t="n">
+        <v>5.98</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1376330968</v>
+      </c>
+      <c r="I18" t="n">
         <v>25269</v>
       </c>
-      <c r="J17" t="n">
+      <c r="J18" t="n">
         <v>135104</v>
       </c>
-      <c r="K17" t="n">
+      <c r="K18" t="n">
         <v>-109835</v>
       </c>
-      <c r="L17" t="n">
+      <c r="L18" t="n">
         <v>-2.04</v>
       </c>
-      <c r="M17" t="n">
+      <c r="M18" t="n">
         <v>-0.48</v>
       </c>
-      <c r="N17" t="n">
-        <v>27.59</v>
-      </c>
-      <c r="O17" t="n">
+      <c r="N18" t="n">
+        <v>27.57</v>
+      </c>
+      <c r="O18" t="n">
         <v>18.68</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P18" t="n">
         <v>13.44</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q18" t="n">
         <v>19289</v>
       </c>
-      <c r="R17" t="n">
+      <c r="R18" t="n">
         <v>-5383</v>
       </c>
-      <c r="S17" t="n">
+      <c r="S18" t="n">
         <v>-13606</v>
       </c>
-      <c r="T17" t="n">
+      <c r="T18" t="n">
         <v>13347</v>
       </c>
-      <c r="U17" t="n">
+      <c r="U18" t="n">
         <v>5942</v>
       </c>
-      <c r="V17" t="n">
+      <c r="V18" t="n">
         <v>10853</v>
       </c>
-      <c r="W17" t="n">
+      <c r="W18" t="n">
         <v>7485</v>
       </c>
-      <c r="X17" t="n">
+      <c r="X18" t="n">
         <v>38889</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="Y18" t="n">
         <v>116684</v>
       </c>
-      <c r="Z17" t="n">
+      <c r="Z18" t="n">
         <v>113.75</v>
       </c>
-      <c r="AA17" t="n">
+      <c r="AA18" t="n">
         <v>41667</v>
       </c>
-      <c r="AB17" t="n">
+      <c r="AB18" t="n">
         <v>24406</v>
       </c>
-      <c r="AC17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD17" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE17" t="n">
+      <c r="AC18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE18" t="n">
         <v>11395</v>
       </c>
     </row>

</xml_diff>